<commit_message>
add Abbreviations to Questions$Title
</commit_message>
<xml_diff>
--- a/inst/extdata/tabulate-fruits.xlsx
+++ b/inst/extdata/tabulate-fruits.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" state="visible" r:id="rId3"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="159">
   <si>
     <t xml:space="preserve">var</t>
   </si>
@@ -432,10 +432,13 @@
     <t xml:space="preserve">Checks</t>
   </si>
   <si>
+    <t xml:space="preserve">Q1. Do you like fruits?</t>
+  </si>
+  <si>
     <t xml:space="preserve">cat</t>
   </si>
   <si>
-    <t xml:space="preserve">Which fruits do you like?</t>
+    <t xml:space="preserve">Q2. Which fruits do you like?</t>
   </si>
   <si>
     <t xml:space="preserve">q2_1 q2_2 q2_3 q2_97</t>
@@ -450,7 +453,7 @@
     <t xml:space="preserve">FILTER</t>
   </si>
   <si>
-    <t xml:space="preserve">Please rate on a scale from 1 to 5 how much you like this fruit</t>
+    <t xml:space="preserve">Q3. Please rate on a scale from 1 to 5 how much you like this fruit</t>
   </si>
   <si>
     <t xml:space="preserve">q3_1 q3_2 q3_3 q3_97</t>
@@ -477,10 +480,16 @@
     <t xml:space="preserve">TOP2:(4 THRU 5=100) (1 THRU 5=0)</t>
   </si>
   <si>
+    <t xml:space="preserve">Q4. What's your favorite fruit?</t>
+  </si>
+  <si>
     <t xml:space="preserve">99, -2</t>
   </si>
   <si>
     <t xml:space="preserve">FILTER: Fruits selected in Q2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q5. How many of your favorite fruit do you like to eat?</t>
   </si>
   <si>
     <t xml:space="preserve">(1 THRU 3 = 1) (4,5 = 2) (6 THRU HI = 3)</t>
@@ -1940,102 +1949,102 @@
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="1" t="s">
-        <v>11</v>
+        <v>133</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>63</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="V4" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="AG5" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="1" t="s">
-        <v>29</v>
+        <v>149</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="1" t="s">
-        <v>32</v>
+        <v>152</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>31</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -2059,7 +2068,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B1" s="1" t="n">
         <v>1</v>
@@ -2067,7 +2076,7 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>4</v>
@@ -2075,7 +2084,7 @@
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>999999999</v>

</xml_diff>